<commit_message>
fix(hassiotis): the three models carry only what the paper publishes
The builder seeded its soil from another sample and overwrote nine fields,
so every shipped model inherited that sample's uncertainties
(sigma_gamma 1.2, sigma_c 1.8, sigma_phi 2.744), its stiffness
(E 50,000 kPa, nu 0.4) and its 3 kPa tensile cutoff. Hassiotis et al.
publish none of these, and the limit-equilibrium path reads none of them.

The material is now written out in full, column by column, the way the
Torggler builder writes its own: sigmas zero, t_cut empty, E and nu left
at the template's empty default. All 21 LEM-HASSIOTIS locks pass on the
rebuilt files, and the sample figures redraw identically.

The corpus index no longer signs these three models "probabilistic", so
the skill's reliability row stops listing a deterministic pile problem.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/lem/files/xslope_hassiotis.xlsx
+++ b/docs/lem/files/xslope_hassiotis.xlsx
@@ -5581,15 +5581,9 @@
       <c r="K11" s="3">
         <v>0.0</v>
       </c>
-      <c r="L11" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="M11" s="3">
-        <v>50000.0</v>
-      </c>
-      <c r="N11" s="3">
-        <v>0.4</v>
-      </c>
+      <c r="L11" s="3" t="n"/>
+      <c r="M11" s="3"/>
+      <c r="N11" s="3"/>
       <c r="O11" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -5625,13 +5619,13 @@
         <v>0.0</v>
       </c>
       <c r="AA11" s="3">
-        <v>1.2</v>
+        <v>0.0</v>
       </c>
       <c r="AB11" s="3">
-        <v>1.8</v>
+        <v>0.0</v>
       </c>
       <c r="AC11" s="3">
-        <v>2.744</v>
+        <v>0.0</v>
       </c>
       <c r="AD11" s="3">
         <v>0.0</v>

</xml_diff>